<commit_message>
Add CHIKV campaign-timing x coverage scenario surface
52 start weeks x 10 coverage levels x 2 vaccine arms, against the share of
symptomatic cases averted, to show what the real-world announcement date cost.
Ixchiq was intended as a pre-outbreak prophylactic (2025-W40); in Caldas Novas it
was announced 18 April 2026 = 2026-W16, after the modelled peak. Both timings are
drawn on the surface.

Deterministic at the central parameter set rather than a Monte Carlo: 1,040 cells
re-propagated would obscure the pattern without changing its shape, and the two
reported timings already carry uncertainty in the main results. The epidemic fit
is done once, with FOI and rho fixed, so only the campaign moves between cells.

Writes an intended_vs_actual sheet giving the fold loss in impact at each
coverage level.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/model_calibration.xlsx
+++ b/model_calibration.xlsx
@@ -586,13 +586,13 @@
         </is>
       </c>
       <c r="C6">
-        <v>1.7143</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="D6">
-        <v>1.6163</v>
+        <v>0.3142857142857143</v>
       </c>
       <c r="E6">
-        <v>1.8123</v>
+        <v>0.5428571428571428</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="H6">
-        <v>1.7143</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="J6">
-        <v>0.05</v>
+        <v>0.05830903790087461</v>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
Retain all 1,000 LHS draws: replace the +/-10% fit screen with FIT_TOL
The screen removed 28 of 1,000 draws, all under-predicting because low reporting
combined with a low symptomatic fraction exhausted the susceptible pool. They are
not worse by likelihood -- 24 of the 28 beat the retained median BIC, and the
single best-BIC draw in the ensemble was among them -- so the screen was
excluding fits the data do not reject.

The tolerance is now a named constant, FIT_TOL, set to Inf to retain everything;
0.10 restores the previous behaviour. attack < 100 stays, being a physical
constraint rather than a fit criterion (no draw ever failed it).

Full CHIKV chain re-run: lhs -> engine -> costs -> outputs -> owsa -> combined.
MAYV needs no re-run: caldas_beta_season.rds comes from the point-estimate fit,
not the ensemble, and is byte-identical after the change.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/model_calibration.xlsx
+++ b/model_calibration.xlsx
@@ -586,34 +586,34 @@
         </is>
       </c>
       <c r="C6">
-        <v>0.4285714285714285</v>
+        <v>0.4481253468959464</v>
       </c>
       <c r="D6">
-        <v>0.3142857142857143</v>
+        <v>0.3428571428571429</v>
       </c>
       <c r="E6">
-        <v>0.5428571428571428</v>
+        <v>0.5857142857142856</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>lognormal</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>α</t>
+          <t>meanlog</t>
         </is>
       </c>
       <c r="H6">
-        <v>0.4285714285714285</v>
+        <v>-0.8026822935232323</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>β</t>
+          <t>sdlog</t>
         </is>
       </c>
       <c r="J6">
-        <v>0.05830903790087461</v>
+        <v>0.1366117949888679</v>
       </c>
     </row>
     <row r="7">

</xml_diff>